<commit_message>
feat: complete Google Maps navigation, Parent Mode, admin dropdowns, and UI refinements
</commit_message>
<xml_diff>
--- a/data/feedback.xlsx
+++ b/data/feedback.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,6 +448,402 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FB0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>20:01:07</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Helpful</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PLACEMENTS</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>verify-session-123</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FB0002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>20:05:09</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Helpful</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PLACEMENTS</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>verify-session-123</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FB0003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>20:19:31</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Helpful</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>PLACEMENTS</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>verify-session-123</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>FB0004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>20:20:50</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Helpful</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ADMISSIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>FB0005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>20:21:42</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Helpful</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>FACILITIES</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>FB0006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>21:59:39</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Helpful</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>PLACEMENTS</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>verify-session-123</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>FB0007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>22:18:20</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Helpful</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>PLACEMENTS</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>verify-session-123</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>FB0008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>23:26:54</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Helpful</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>CONTACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FB0009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>23:47:59</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Helpful</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>PLACEMENTS</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>verify-session-123</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>FB0010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>00:01:30</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Helpful</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>PLACEMENTS</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>verify-session-123</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>FB0011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>01:38:33</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Unhelpful</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ADMISSIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>FB0012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>07:23:28</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Helpful</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>PLACEMENTS</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>verify-session-123</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>FB0013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>07:58:16</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Helpful</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>PLACEMENTS</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>verify-session-123</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>